<commit_message>
defect-hub: master workbook (5 records)
</commit_message>
<xml_diff>
--- a/master/CleanCore_Defects_Master.xlsx
+++ b/master/CleanCore_Defects_Master.xlsx
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="57">
   <si>
     <t>Customer</t>
   </si>
@@ -243,31 +243,43 @@
     <t>mkarthik@smartshift.com</t>
   </si>
   <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>attachments/samples/st22_cast_dump.png|attachments/samples/analysis_cast_error.docx</t>
+  </si>
+  <si>
+    <t>JAIT-12</t>
+  </si>
+  <si>
+    <t>PROCESSED</t>
+  </si>
+  <si>
+    <t>2026-10-29T08:14:51.014Z</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>CDS view ZI_SalesDocItem returns duplicate rows after VBAP replacement</t>
+  </si>
+  <si>
+    <t>After replacing direct SELECT on VBAP with CDS view ZI_SalesDocItem the item count doubles for orders with multiple schedule lines (VBEP). Join cardinality on _ScheduleLine is MANY instead of ONE.</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
     <t>In Progress</t>
   </si>
   <si>
-    <t>attachments/samples/st22_cast_dump.png|attachments/samples/analysis_cast_error.docx</t>
-  </si>
-  <si>
-    <t/>
+    <t>attachments/samples/cds_duplicate_rows.png|attachments/samples/cds_row_counts.xlsx</t>
   </si>
   <si>
     <t>PENDING</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>CDS view ZI_SalesDocItem returns duplicate rows after VBAP replacement</t>
-  </si>
-  <si>
-    <t>After replacing direct SELECT on VBAP with CDS view ZI_SalesDocItem the item count doubles for orders with multiple schedule lines (VBEP). Join cardinality on _ScheduleLine is MANY instead of ONE.</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>attachments/samples/cds_duplicate_rows.png|attachments/samples/cds_row_counts.xlsx</t>
   </si>
   <si>
     <t>P&amp;G</t>
@@ -846,16 +858,16 @@
         <v>32</v>
       </c>
       <c r="P2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
       <c r="R2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -872,10 +884,10 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G3" t="s">
         <v>25</v>
@@ -884,7 +896,7 @@
         <v>26</v>
       </c>
       <c r="I3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J3" t="s">
         <v>28</v>
@@ -893,33 +905,33 @@
         <v>28</v>
       </c>
       <c r="L3" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="M3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="N3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="O3" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="P3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
       <c r="R3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -931,19 +943,19 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H4" t="s">
         <v>26</v>
       </c>
       <c r="I4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="J4" t="s">
         <v>28</v>
@@ -952,33 +964,33 @@
         <v>28</v>
       </c>
       <c r="L4" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="M4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="N4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="O4" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="P4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
       <c r="R4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -990,10 +1002,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F5" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G5" t="s">
         <v>25</v>
@@ -1002,7 +1014,7 @@
         <v>26</v>
       </c>
       <c r="I5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="J5" t="s">
         <v>28</v>
@@ -1011,33 +1023,33 @@
         <v>28</v>
       </c>
       <c r="L5" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="M5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="N5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="O5" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="P5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
       <c r="R5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -1049,19 +1061,19 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="H6" t="s">
         <v>26</v>
       </c>
       <c r="I6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="J6" t="s">
         <v>28</v>
@@ -1070,28 +1082,28 @@
         <v>28</v>
       </c>
       <c r="L6" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="M6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="N6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="O6" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="P6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
       <c r="R6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
defect-hub: master workbook (7 records)
</commit_message>
<xml_diff>
--- a/master/CleanCore_Defects_Master.xlsx
+++ b/master/CleanCore_Defects_Master.xlsx
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="64">
   <si>
     <t>Customer</t>
   </si>
@@ -334,6 +334,18 @@
   </si>
   <si>
     <t>attachments/samples/mrp_type_comparison.xlsx|attachments/samples/analysis_cast_error.docx</t>
+  </si>
+  <si>
+    <t>some of CDS views authorization Issue</t>
+  </si>
+  <si>
+    <t>Almost 10 CDS view we faced authorization issue</t>
+  </si>
+  <si>
+    <t>Clean Core analysis</t>
+  </si>
+  <si>
+    <t>Need to run end to end analysis of Clean core</t>
   </si>
 </sst>
 </file>
@@ -738,7 +750,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:S8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1115,6 +1127,124 @@
         <v>35</v>
       </c>
     </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G7" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" t="s">
+        <v>28</v>
+      </c>
+      <c r="K7" t="s">
+        <v>28</v>
+      </c>
+      <c r="L7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M7" t="s">
+        <v>30</v>
+      </c>
+      <c r="N7" t="s">
+        <v>34</v>
+      </c>
+      <c r="O7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P7" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7" t="s">
+        <v>34</v>
+      </c>
+      <c r="S7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" t="s">
+        <v>62</v>
+      </c>
+      <c r="F8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" t="s">
+        <v>26</v>
+      </c>
+      <c r="I8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J8" t="s">
+        <v>28</v>
+      </c>
+      <c r="K8" t="s">
+        <v>28</v>
+      </c>
+      <c r="L8" t="s">
+        <v>39</v>
+      </c>
+      <c r="M8" t="s">
+        <v>40</v>
+      </c>
+      <c r="N8" t="s">
+        <v>34</v>
+      </c>
+      <c r="O8" t="s">
+        <v>41</v>
+      </c>
+      <c r="P8" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S8" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
defect-hub: master workbook (9 records)
</commit_message>
<xml_diff>
--- a/master/CleanCore_Defects_Master.xlsx
+++ b/master/CleanCore_Defects_Master.xlsx
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="70">
   <si>
     <t>Customer</t>
   </si>
@@ -352,6 +352,18 @@
   </si>
   <si>
     <t>Need to run end to end analysis of Clean core</t>
+  </si>
+  <si>
+    <t>Security issue causing in CRUD</t>
+  </si>
+  <si>
+    <t>One of the customer facing Security Issue</t>
+  </si>
+  <si>
+    <t>Duplicate records showing in excel</t>
+  </si>
+  <si>
+    <t>Shows Duplicate entries on multiple projects</t>
   </si>
 </sst>
 </file>
@@ -756,7 +768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:S10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1251,6 +1263,124 @@
         <v>35</v>
       </c>
     </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" t="s">
+        <v>26</v>
+      </c>
+      <c r="I9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" t="s">
+        <v>28</v>
+      </c>
+      <c r="K9" t="s">
+        <v>28</v>
+      </c>
+      <c r="L9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" t="s">
+        <v>30</v>
+      </c>
+      <c r="N9" t="s">
+        <v>34</v>
+      </c>
+      <c r="O9" t="s">
+        <v>41</v>
+      </c>
+      <c r="P9" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9" t="s">
+        <v>34</v>
+      </c>
+      <c r="S9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" t="s">
+        <v>38</v>
+      </c>
+      <c r="J10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K10" t="s">
+        <v>28</v>
+      </c>
+      <c r="L10" t="s">
+        <v>39</v>
+      </c>
+      <c r="M10" t="s">
+        <v>40</v>
+      </c>
+      <c r="N10" t="s">
+        <v>34</v>
+      </c>
+      <c r="O10" t="s">
+        <v>41</v>
+      </c>
+      <c r="P10" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10" t="s">
+        <v>34</v>
+      </c>
+      <c r="S10" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>